<commit_message>
docs: work of mercy added to the spreadsheet
</commit_message>
<xml_diff>
--- a/inventory_cvbc.xlsx
+++ b/inventory_cvbc.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Odyce\Documents\Work_Doc\Archipelago\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Odyce\Documents\Work_Doc\Archipelago\Belmont_s_Curse_APWorld\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92B4A6B-726D-4CC3-9FDA-21CE74B9D8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C475196-FAD2-4107-9FDA-6C45705C384E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="568" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="568" firstSheet="1" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Help" sheetId="1" r:id="rId1"/>
@@ -33,11 +33,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">Enemies!$A$2:$E$500</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ID Range'!$A$2:$F$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Items!$A$2:$K$251</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Locations!$A$2:$K$493</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Locations!$A$2:$K$492</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Progressive Weapons'!$A$2:$E$500</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">Status!$A$2:$F$500</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Total!$A$2:$D$501</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Works of Mercy'!$A$2:$I$499</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Works of Mercy'!$A$2:$G$499</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5047" uniqueCount="1470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5399" uniqueCount="1605">
   <si>
     <t>Inventory – Castlevania: Belmont's Curse (APWorld cvbc)</t>
   </si>
@@ -4343,12 +4343,6 @@
     <t>Challenge (condition)</t>
   </si>
   <si>
-    <t>Card(s) required to do it</t>
-  </si>
-  <si>
-    <t>Other prerequisites</t>
-  </si>
-  <si>
     <t>Upgrade 1</t>
   </si>
   <si>
@@ -4470,13 +4464,424 @@
   </si>
   <si>
     <t>• Jeanne d'Arc and Aliénor d'Aquitaine keep their French names on purpose (client and AP messages). Please respect this little quirk of mine</t>
+  </si>
+  <si>
+    <t>WOM - Cursed Flame 1</t>
+  </si>
+  <si>
+    <t>WOM - Absolution 1</t>
+  </si>
+  <si>
+    <t>WOM - Absolution 2</t>
+  </si>
+  <si>
+    <t>WOM - Absolution 3</t>
+  </si>
+  <si>
+    <t>WOM - Holy Cross 1</t>
+  </si>
+  <si>
+    <t>WOM - Holy Cross 2</t>
+  </si>
+  <si>
+    <t>WOM - Holy Cross 3</t>
+  </si>
+  <si>
+    <t>WOM - Infernal Pyre 1</t>
+  </si>
+  <si>
+    <t>WOM - Infernal Pyre 2</t>
+  </si>
+  <si>
+    <t>WOM - Infernal Pyre 3</t>
+  </si>
+  <si>
+    <t>WOM - Petrifying Gaze 1</t>
+  </si>
+  <si>
+    <t>WOM - Petrifying Gaze 2</t>
+  </si>
+  <si>
+    <t>WOM - Fist of Talos 1</t>
+  </si>
+  <si>
+    <t>WOM - Fist of Talos 2</t>
+  </si>
+  <si>
+    <t>WOM - Fist of Talos 3</t>
+  </si>
+  <si>
+    <t>WOM - Masterpiece 1</t>
+  </si>
+  <si>
+    <t>WOM - Masterpiece 2</t>
+  </si>
+  <si>
+    <t>WOM - Masterpiece 3</t>
+  </si>
+  <si>
+    <t>WOM - Bloody Spikes 1</t>
+  </si>
+  <si>
+    <t>WOM - Bloody Spikes 2</t>
+  </si>
+  <si>
+    <t>WOM - Bloody Spikes 3</t>
+  </si>
+  <si>
+    <t>WOM - Soul Harvest 1</t>
+  </si>
+  <si>
+    <t>WOM - Soul Harvest 2</t>
+  </si>
+  <si>
+    <t>WOM - Soul Harvest 3</t>
+  </si>
+  <si>
+    <t>WOM - Wheel of Chaos 1</t>
+  </si>
+  <si>
+    <t>WOM - Wheel of Chaos 2</t>
+  </si>
+  <si>
+    <t>WOM - Wheel of Chaos 3</t>
+  </si>
+  <si>
+    <t>WOM - Freezing Path 1</t>
+  </si>
+  <si>
+    <t>WOM - Freezing Path 2</t>
+  </si>
+  <si>
+    <t>WOM - Chronomantic Dive 1</t>
+  </si>
+  <si>
+    <t>WOM - Chronomantic Dive 2</t>
+  </si>
+  <si>
+    <t>WOM - Life Drain 1</t>
+  </si>
+  <si>
+    <t>WOM - Life Drain 2</t>
+  </si>
+  <si>
+    <t>WOM - Life Drain 3</t>
+  </si>
+  <si>
+    <t>WOM - Stained-Glass Shield 1</t>
+  </si>
+  <si>
+    <t>WOM - Stained-Glass Shield 2</t>
+  </si>
+  <si>
+    <t>WOM - Stained-Glass Shield 3</t>
+  </si>
+  <si>
+    <t>WOM - Chains of Justice 1</t>
+  </si>
+  <si>
+    <t>WOM - Chains of Justice 2</t>
+  </si>
+  <si>
+    <t>WOM - Chains of Justice 3</t>
+  </si>
+  <si>
+    <t>WOM - Mirror Walk 1</t>
+  </si>
+  <si>
+    <t>WOM - Mirror Walk 2</t>
+  </si>
+  <si>
+    <t>WOM - Mirror Walk 3</t>
+  </si>
+  <si>
+    <t>Work of Mercy of Tarot : The Fallen</t>
+  </si>
+  <si>
+    <t>Work of Mercy of Tarot : The Prophetess</t>
+  </si>
+  <si>
+    <t>Work of Mercy of Tarot : The Occultist</t>
+  </si>
+  <si>
+    <t>Work of Mercy of Tarot : The Zealot</t>
+  </si>
+  <si>
+    <t>Work of Mercy of Tarot : The Brittle King</t>
+  </si>
+  <si>
+    <t>Tarot : The Justice</t>
+  </si>
+  <si>
+    <t>Hit 20 times with this spell.</t>
+  </si>
+  <si>
+    <t>Kill 4 enemies with one cast of this spell, 5 times.</t>
+  </si>
+  <si>
+    <t>Explore 85% of the whole map.</t>
+  </si>
+  <si>
+    <t>Heal back to full life using this spell 10 times.</t>
+  </si>
+  <si>
+    <t>Find 3 different whip-type weapons.</t>
+  </si>
+  <si>
+    <t>Kill 5 enemies with the same cross (not necessarily at the same time).</t>
+  </si>
+  <si>
+    <t>Kill 10 enemies with a whip attack.</t>
+  </si>
+  <si>
+    <t>Successfully parry 15 attacks with the Holy Light.</t>
+  </si>
+  <si>
+    <t>Reach a sacred place so Joan can pray.</t>
+  </si>
+  <si>
+    <t>Set 5 enemies on fire at the same time.</t>
+  </si>
+  <si>
+    <t>Petrify an enemy carrying a shield with Medusa’s Spell. Not again, Perseus!</t>
+  </si>
+  <si>
+    <t>Kill 25 enemies from fall damage directly after petrifying them in the air.</t>
+  </si>
+  <si>
+    <t>Kill 3 enemies with one fist.</t>
+  </si>
+  <si>
+    <t>Kill 10 airborne enemy with a fist as it falls down.</t>
+  </si>
+  <si>
+    <t>Kill 15 enemies with the smash.</t>
+  </si>
+  <si>
+    <t>Kill 30 enemies with the Gargoyle Dive.</t>
+  </si>
+  <si>
+    <t>Cause 5 enemies to fall to their death with the Gargoyle Summoning Stone.</t>
+  </si>
+  <si>
+    <t>Find all the secret zones in the Main Hall.</t>
+  </si>
+  <si>
+    <t>Kill 25 enemies from bleed-effect damage.</t>
+  </si>
+  <si>
+    <t>Find 2 different dual blade-type weapons.</t>
+  </si>
+  <si>
+    <t>Cause an enemy to bleed continuously for 10 seconds.</t>
+  </si>
+  <si>
+    <t>Complete the hidden puzzle in Notre Dame.</t>
+  </si>
+  <si>
+    <t>Kill 44 skeletons (of any sort).</t>
+  </si>
+  <si>
+    <t>Kill 4 enemies with the same cast of Death’s spell.</t>
+  </si>
+  <si>
+    <t>Have the wheel spin for 15 seconds without interruption.</t>
+  </si>
+  <si>
+    <t>Kill 5 different enemies with one wheel.</t>
+  </si>
+  <si>
+    <t>Spend 1000 mana points on recasts of this spell.</t>
+  </si>
+  <si>
+    <t>Kill 25 enemies by breaking them out of freeze.</t>
+  </si>
+  <si>
+    <t>Pass through 5 enemies in 3 seconds.</t>
+  </si>
+  <si>
+    <t>Kill 20 enemies while in slow motion.</t>
+  </si>
+  <si>
+    <t>Explore all rooms of Clock Tower.</t>
+  </si>
+  <si>
+    <t>Drain an enemy for 5 seconds straight without interruption.</t>
+  </si>
+  <si>
+    <t>Explore all rooms of Hall of Mirrors.</t>
+  </si>
+  <si>
+    <t>Kill 25 enemies with the life drain.</t>
+  </si>
+  <si>
+    <t>Absorb an attack that would otherwise be fatal thanks to Arthur's spell.</t>
+  </si>
+  <si>
+    <t>Kill 25 Haunted Armor.</t>
+  </si>
+  <si>
+    <t>Kill 3 enemies with a single attack.</t>
+  </si>
+  <si>
+    <t>Chain 4 enemies at once.</t>
+  </si>
+  <si>
+    <t>Kill 25 chained enemies.</t>
+  </si>
+  <si>
+    <t>Upgrade your maximum health and mana 5 times each.</t>
+  </si>
+  <si>
+    <t>Use 34 Save Rooms.</t>
+  </si>
+  <si>
+    <t>Heal 1000 of health with this spell.</t>
+  </si>
+  <si>
+    <t>Kill 5 enemies within 3 seconds of dodging their attacks with teleportation.</t>
+  </si>
+  <si>
+    <t>Fires a bigger gireball that slightly pushes back its target.</t>
+  </si>
+  <si>
+    <t>If the spell is cast while Rose is at full health, deals 50% more damage.</t>
+  </si>
+  <si>
+    <t>If the spell hits only one target, ignites it.</t>
+  </si>
+  <si>
+    <t>If the spell kills at least 4 enemies, heals Rose back to full health.</t>
+  </si>
+  <si>
+    <t>You can throw a second cross.</t>
+  </si>
+  <si>
+    <t>The cross inflicts more damage the farther it is from Rose.</t>
+  </si>
+  <si>
+    <t>Catching the returning cross lets Rose regain 10% of the spell's mana cast for each time an enemy was hit, up to a maximum of 60%.</t>
+  </si>
+  <si>
+    <t>Regain 25% of the spell's mana cost for each enemy hit by the central explosion, starting with the second enemy.</t>
+  </si>
+  <si>
+    <t>Enemies hit by Joan's spell are thrown high in the air.</t>
+  </si>
+  <si>
+    <t>Hitting an enemy with a weapon prolong the fire on them.</t>
+  </si>
+  <si>
+    <t>Killing a petrified enemy restores a quantity of mana equivalent to half the cost of Medusa's spell.</t>
+  </si>
+  <si>
+    <t>The closer the targets affected by this spell are to Rose, the longer they remain petrified, and the more hits it takes to break the petrification.</t>
+  </si>
+  <si>
+    <t>The fist deals 75% more damage to enemies suffering fro control effects.</t>
+  </si>
+  <si>
+    <t>The earthquake is more powerful and unleashes 1 second later.</t>
+  </si>
+  <si>
+    <t>The fists is covered in damage-dealing spikes that hit enemies even after hiting the ground.</t>
+  </si>
+  <si>
+    <t>Summons an additional Gargoyle</t>
+  </si>
+  <si>
+    <t>Rose heals every time the Gargoyle's fire ball hits an enemy.</t>
+  </si>
+  <si>
+    <t>Killing at least one enemy with the Gargoyle Dive prevents the Gargoyle's destruction.</t>
+  </si>
+  <si>
+    <t>Applying the bleeding effect to an already bleeding enemy deals instant damage to it.</t>
+  </si>
+  <si>
+    <t>Heals Rose 2% of her max health every time an enemy dies from bleeding.</t>
+  </si>
+  <si>
+    <t>Bleeding enemies are slower and deal 25% less damage to Rose.</t>
+  </si>
+  <si>
+    <t>If this spell only hits one enemy, Rose heals 4% of her maximum health.</t>
+  </si>
+  <si>
+    <t>If a sickle kills an enemy, it splits into 4 new sickles.</t>
+  </si>
+  <si>
+    <t>Each sickle that hits an enemy restores 25% of the spell's mana cost.</t>
+  </si>
+  <si>
+    <t>The spell can be cast using health if Rose does not have enough mana and will deal 50% more damage.</t>
+  </si>
+  <si>
+    <t>Mammon's spell deals increased damage each time it is cast. This bonus resets if the spell is not recast while active.</t>
+  </si>
+  <si>
+    <t>Every time the player recasts the spell, there is a 1/8 chance of triggering a random effect.</t>
+  </si>
+  <si>
+    <t>At the end of the spell effect, a wave of frost bursts around Rose that freezes enemies within a radius of 5 meters.</t>
+  </si>
+  <si>
+    <t>Passing through an enemy increases your speed by 10% for a maximum of 5 times. Can only trigger once on the same enemy.</t>
+  </si>
+  <si>
+    <t>The time slow effect is longer.</t>
+  </si>
+  <si>
+    <t>Creates a bigger explosion if Rose dives from a high enough position.</t>
+  </si>
+  <si>
+    <t>The drain deals bonus damage if Rose is at full health when it ticks.</t>
+  </si>
+  <si>
+    <t>Getting hit while holding this spell doesn't interrupt it.</t>
+  </si>
+  <si>
+    <t>The spell targets the 2 nearest enemies instead of just one.</t>
+  </si>
+  <si>
+    <t>The spell's magic shield can absorb 1 additional attacks before it breaks.</t>
+  </si>
+  <si>
+    <t>Each time Rose takes damage (with or without an active magic shield), a shard if glass is launched at the nearest enemy.</t>
+  </si>
+  <si>
+    <t>When Rose is struck during an attackm damage received is reduced by 50% and her attack continues uninterrupted.</t>
+  </si>
+  <si>
+    <t>Chained enemies are also rendered incapable of performing any action.</t>
+  </si>
+  <si>
+    <t>Killing a chained target chains a nearby target.</t>
+  </si>
+  <si>
+    <t>Chaining an enemy with less than 20% of their maximum health instantly kills them.</t>
+  </si>
+  <si>
+    <t>If Rose uses teleportation without losing life since the mirror is placed, she regains 80% of the consumed mana.</t>
+  </si>
+  <si>
+    <t>Rose deals significant damage to enemies in the path of the teleportation.</t>
+  </si>
+  <si>
+    <t>Receiving a fatal blow while a mirror is active prevents death and activates teleportation. Can only be activated once but can recharged when Rose interacts with a Save Room.</t>
+  </si>
+  <si>
+    <t>//</t>
+  </si>
+  <si>
+    <t>Can be completed before getting the card</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4550,6 +4955,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -4583,7 +4994,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4630,6 +5041,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5085,7 +5499,7 @@
     </row>
     <row r="40" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>1469</v>
+        <v>1467</v>
       </c>
     </row>
   </sheetData>
@@ -5107,21 +5521,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>1433</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>1434</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>1435</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>1436</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>1437</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>58</v>
@@ -5129,10 +5543,10 @@
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>1438</v>
+        <v>1436</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>1439</v>
+        <v>1437</v>
       </c>
       <c r="C3" s="15" t="s">
         <v>1282</v>
@@ -5168,24 +5582,24 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>1440</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
+        <v>1439</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>1441</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>1442</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>1443</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>1444</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>1445</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>58</v>
@@ -5193,10 +5607,10 @@
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>1446</v>
+        <v>1444</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>1447</v>
+        <v>1445</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15" t="s">
@@ -5207,10 +5621,10 @@
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1448</v>
+        <v>1446</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1449</v>
+        <v>1447</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -5224,10 +5638,10 @@
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1450</v>
+        <v>1448</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1451</v>
+        <v>1449</v>
       </c>
       <c r="C5">
         <v>8</v>
@@ -5241,10 +5655,10 @@
     </row>
     <row r="6" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1452</v>
+        <v>1450</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>1453</v>
+        <v>1451</v>
       </c>
       <c r="C6">
         <v>3</v>
@@ -5258,10 +5672,10 @@
     </row>
     <row r="7" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1454</v>
+        <v>1452</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1455</v>
+        <v>1453</v>
       </c>
       <c r="C7">
         <v>4</v>
@@ -5275,10 +5689,10 @@
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1456</v>
+        <v>1454</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1457</v>
+        <v>1455</v>
       </c>
       <c r="C8">
         <v>3</v>
@@ -5292,10 +5706,10 @@
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1459</v>
+        <v>1457</v>
       </c>
       <c r="C9">
         <v>7</v>
@@ -5825,12 +6239,12 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>1460</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>1461</v>
+        <v>1459</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>51</v>
@@ -5847,13 +6261,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>1462</v>
+        <v>1460</v>
       </c>
       <c r="B3" s="15">
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>1463</v>
+        <v>1461</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="16"/>
@@ -5872,7 +6286,7 @@
         <v>148</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>1464</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -6085,7 +6499,7 @@
         <v>182</v>
       </c>
       <c r="D19" t="s">
-        <v>1465</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -6183,7 +6597,7 @@
         <v>198</v>
       </c>
       <c r="D26" t="s">
-        <v>1466</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -6197,7 +6611,7 @@
         <v>200</v>
       </c>
       <c r="D27" t="s">
-        <v>1467</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -6256,7 +6670,7 @@
         <v>209</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>1468</v>
+        <v>1466</v>
       </c>
       <c r="E31" s="3"/>
     </row>
@@ -6306,7 +6720,7 @@
         <v>42</v>
       </c>
       <c r="C3" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A3)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A3)</f>
         <v>42</v>
       </c>
       <c r="D3" s="6">
@@ -6323,7 +6737,7 @@
         <v>28</v>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A4)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A4)</f>
         <v>28</v>
       </c>
       <c r="D4" s="6">
@@ -6340,7 +6754,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A5)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A5)</f>
         <v>40</v>
       </c>
       <c r="D5" s="6">
@@ -6357,7 +6771,7 @@
         <v>16</v>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A6)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A6)</f>
         <v>16</v>
       </c>
       <c r="D6" s="6">
@@ -6374,7 +6788,7 @@
         <v>76</v>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A7)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A7)</f>
         <v>76</v>
       </c>
       <c r="D7" s="6">
@@ -6388,11 +6802,11 @@
       </c>
       <c r="B8" s="6">
         <f>SUMIFS(Items!$E$3:$E$400,Items!$B$3:$B$400,A8)</f>
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A8)</f>
-        <v>44</v>
+        <f>COUNTIF(Locations!$C$3:$C$499,A8)</f>
+        <v>43</v>
       </c>
       <c r="D8" s="6">
         <f t="shared" si="0"/>
@@ -6408,7 +6822,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A9)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A9)</f>
         <v>19</v>
       </c>
       <c r="D9" s="6">
@@ -6425,7 +6839,7 @@
         <v>147</v>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIF(Locations!$C$3:$C$500,A10)</f>
+        <f>COUNTIF(Locations!$C$3:$C$499,A10)</f>
         <v>147</v>
       </c>
       <c r="D10" s="6">
@@ -6439,11 +6853,11 @@
       </c>
       <c r="B11" s="5">
         <f>SUM(B3:B10)</f>
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C11" s="5">
         <f>SUM(C3:C10)</f>
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D11" s="5">
         <f>SUM(D3:D10)</f>
@@ -10029,6 +10443,9 @@
       <c r="I142" s="22">
         <v>7006003</v>
       </c>
+      <c r="K142" s="1" t="s">
+        <v>1511</v>
+      </c>
     </row>
     <row r="143" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
@@ -10064,7 +10481,7 @@
         <v>43</v>
       </c>
       <c r="E144">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F144" t="s">
         <v>60</v>
@@ -10077,6 +10494,9 @@
       </c>
       <c r="I144" s="22">
         <v>7006005</v>
+      </c>
+      <c r="K144" s="1" t="s">
+        <v>1512</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -10153,6 +10573,9 @@
       <c r="I147" s="22">
         <v>7006008</v>
       </c>
+      <c r="K147" s="1" t="s">
+        <v>1513</v>
+      </c>
     </row>
     <row r="148" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
@@ -10254,6 +10677,9 @@
       <c r="I151" s="22">
         <v>7006012</v>
       </c>
+      <c r="K151" s="1" t="s">
+        <v>1514</v>
+      </c>
     </row>
     <row r="152" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
@@ -10302,6 +10728,9 @@
       </c>
       <c r="I153" s="22">
         <v>7006014</v>
+      </c>
+      <c r="K153" s="1" t="s">
+        <v>1515</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -11195,7 +11624,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L414"/>
+  <dimension ref="A1:L413"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -22909,6 +23338,9 @@
       </c>
     </row>
     <row r="367" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A367" t="s">
+        <v>1468</v>
+      </c>
       <c r="B367" t="s">
         <v>1279</v>
       </c>
@@ -22921,6 +23353,9 @@
       <c r="E367" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G367" s="1" t="s">
+        <v>293</v>
+      </c>
       <c r="I367" s="23">
         <v>7106001</v>
       </c>
@@ -22929,6 +23364,9 @@
       </c>
     </row>
     <row r="368" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A368" t="s">
+        <v>1469</v>
+      </c>
       <c r="B368" t="s">
         <v>1279</v>
       </c>
@@ -22941,6 +23379,9 @@
       <c r="E368" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G368" s="1" t="s">
+        <v>296</v>
+      </c>
       <c r="I368" s="23">
         <v>7106002</v>
       </c>
@@ -22948,7 +23389,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="369" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A369" t="s">
+        <v>1470</v>
+      </c>
       <c r="B369" t="s">
         <v>1279</v>
       </c>
@@ -22961,6 +23405,9 @@
       <c r="E369" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G369" s="1" t="s">
+        <v>296</v>
+      </c>
       <c r="I369" s="23">
         <v>7106003</v>
       </c>
@@ -22968,7 +23415,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="370" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A370" t="s">
+        <v>1471</v>
+      </c>
       <c r="B370" t="s">
         <v>1279</v>
       </c>
@@ -22981,6 +23431,9 @@
       <c r="E370" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G370" s="1" t="s">
+        <v>296</v>
+      </c>
       <c r="I370" s="23">
         <v>7106004</v>
       </c>
@@ -22988,7 +23441,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="371" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A371" t="s">
+        <v>1472</v>
+      </c>
       <c r="B371" t="s">
         <v>1279</v>
       </c>
@@ -23001,6 +23457,9 @@
       <c r="E371" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G371" s="1" t="s">
+        <v>301</v>
+      </c>
       <c r="I371" s="23">
         <v>7106005</v>
       </c>
@@ -23008,7 +23467,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="372" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A372" t="s">
+        <v>1473</v>
+      </c>
       <c r="B372" t="s">
         <v>1279</v>
       </c>
@@ -23021,6 +23483,9 @@
       <c r="E372" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G372" s="1" t="s">
+        <v>301</v>
+      </c>
       <c r="I372" s="23">
         <v>7106006</v>
       </c>
@@ -23028,7 +23493,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="373" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A373" t="s">
+        <v>1474</v>
+      </c>
       <c r="B373" t="s">
         <v>1279</v>
       </c>
@@ -23041,6 +23509,9 @@
       <c r="E373" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G373" s="1" t="s">
+        <v>301</v>
+      </c>
       <c r="I373" s="23">
         <v>7106007</v>
       </c>
@@ -23048,7 +23519,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="374" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A374" t="s">
+        <v>1475</v>
+      </c>
       <c r="B374" t="s">
         <v>1279</v>
       </c>
@@ -23061,6 +23535,9 @@
       <c r="E374" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G374" s="1" t="s">
+        <v>303</v>
+      </c>
       <c r="I374" s="23">
         <v>7106008</v>
       </c>
@@ -23068,7 +23545,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="375" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A375" t="s">
+        <v>1476</v>
+      </c>
       <c r="B375" t="s">
         <v>1279</v>
       </c>
@@ -23081,6 +23561,9 @@
       <c r="E375" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G375" s="1" t="s">
+        <v>303</v>
+      </c>
       <c r="I375" s="23">
         <v>7106009</v>
       </c>
@@ -23088,7 +23571,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="376" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A376" t="s">
+        <v>1477</v>
+      </c>
       <c r="B376" t="s">
         <v>1279</v>
       </c>
@@ -23101,6 +23587,9 @@
       <c r="E376" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G376" s="1" t="s">
+        <v>303</v>
+      </c>
       <c r="I376" s="23">
         <v>7106010</v>
       </c>
@@ -23108,7 +23597,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="377" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A377" t="s">
+        <v>1478</v>
+      </c>
       <c r="B377" t="s">
         <v>1279</v>
       </c>
@@ -23121,6 +23613,9 @@
       <c r="E377" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G377" s="1" t="s">
+        <v>307</v>
+      </c>
       <c r="I377" s="23">
         <v>7106011</v>
       </c>
@@ -23128,7 +23623,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="378" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A378" t="s">
+        <v>1479</v>
+      </c>
       <c r="B378" t="s">
         <v>1279</v>
       </c>
@@ -23141,6 +23639,9 @@
       <c r="E378" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G378" s="1" t="s">
+        <v>307</v>
+      </c>
       <c r="I378" s="23">
         <v>7106012</v>
       </c>
@@ -23148,7 +23649,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="379" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A379" t="s">
+        <v>1480</v>
+      </c>
       <c r="B379" t="s">
         <v>1279</v>
       </c>
@@ -23161,6 +23665,9 @@
       <c r="E379" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G379" s="1" t="s">
+        <v>310</v>
+      </c>
       <c r="I379" s="23">
         <v>7106013</v>
       </c>
@@ -23168,7 +23675,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="380" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A380" t="s">
+        <v>1481</v>
+      </c>
       <c r="B380" t="s">
         <v>1279</v>
       </c>
@@ -23181,6 +23691,9 @@
       <c r="E380" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G380" s="1" t="s">
+        <v>310</v>
+      </c>
       <c r="I380" s="23">
         <v>7106014</v>
       </c>
@@ -23188,7 +23701,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="381" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A381" t="s">
+        <v>1482</v>
+      </c>
       <c r="B381" t="s">
         <v>1279</v>
       </c>
@@ -23201,6 +23717,9 @@
       <c r="E381" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G381" s="1" t="s">
+        <v>310</v>
+      </c>
       <c r="I381" s="23">
         <v>7106015</v>
       </c>
@@ -23208,7 +23727,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="382" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A382" t="s">
+        <v>1483</v>
+      </c>
       <c r="B382" t="s">
         <v>1279</v>
       </c>
@@ -23221,6 +23743,9 @@
       <c r="E382" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G382" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="I382" s="23">
         <v>7106016</v>
       </c>
@@ -23228,7 +23753,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="383" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A383" t="s">
+        <v>1484</v>
+      </c>
       <c r="B383" t="s">
         <v>1279</v>
       </c>
@@ -23241,6 +23769,9 @@
       <c r="E383" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G383" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="I383" s="23">
         <v>7106017</v>
       </c>
@@ -23248,7 +23779,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="384" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A384" t="s">
+        <v>1485</v>
+      </c>
       <c r="B384" t="s">
         <v>1279</v>
       </c>
@@ -23261,6 +23795,9 @@
       <c r="E384" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G384" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="I384" s="23">
         <v>7106018</v>
       </c>
@@ -23268,7 +23805,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="385" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A385" t="s">
+        <v>1486</v>
+      </c>
       <c r="B385" t="s">
         <v>1279</v>
       </c>
@@ -23281,6 +23821,9 @@
       <c r="E385" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G385" s="1" t="s">
+        <v>318</v>
+      </c>
       <c r="I385" s="23">
         <v>7106019</v>
       </c>
@@ -23288,7 +23831,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="386" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>1487</v>
+      </c>
       <c r="B386" t="s">
         <v>1279</v>
       </c>
@@ -23301,6 +23847,9 @@
       <c r="E386" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G386" s="1" t="s">
+        <v>318</v>
+      </c>
       <c r="I386" s="23">
         <v>7106020</v>
       </c>
@@ -23308,7 +23857,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="387" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>1488</v>
+      </c>
       <c r="B387" t="s">
         <v>1279</v>
       </c>
@@ -23321,6 +23873,9 @@
       <c r="E387" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G387" s="1" t="s">
+        <v>318</v>
+      </c>
       <c r="I387" s="23">
         <v>7106021</v>
       </c>
@@ -23328,7 +23883,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="388" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>1489</v>
+      </c>
       <c r="B388" t="s">
         <v>1279</v>
       </c>
@@ -23341,6 +23899,9 @@
       <c r="E388" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G388" s="1" t="s">
+        <v>320</v>
+      </c>
       <c r="I388" s="23">
         <v>7106022</v>
       </c>
@@ -23348,7 +23909,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="389" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>1490</v>
+      </c>
       <c r="B389" t="s">
         <v>1279</v>
       </c>
@@ -23361,6 +23925,9 @@
       <c r="E389" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G389" s="1" t="s">
+        <v>320</v>
+      </c>
       <c r="I389" s="23">
         <v>7106023</v>
       </c>
@@ -23368,7 +23935,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="390" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>1491</v>
+      </c>
       <c r="B390" t="s">
         <v>1279</v>
       </c>
@@ -23381,6 +23951,9 @@
       <c r="E390" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G390" s="1" t="s">
+        <v>320</v>
+      </c>
       <c r="I390" s="23">
         <v>7106024</v>
       </c>
@@ -23388,7 +23961,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="391" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>1492</v>
+      </c>
       <c r="B391" t="s">
         <v>1279</v>
       </c>
@@ -23401,6 +23977,9 @@
       <c r="E391" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G391" s="1" t="s">
+        <v>324</v>
+      </c>
       <c r="I391" s="23">
         <v>7106025</v>
       </c>
@@ -23408,7 +23987,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="392" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>1493</v>
+      </c>
       <c r="B392" t="s">
         <v>1279</v>
       </c>
@@ -23421,6 +24003,9 @@
       <c r="E392" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G392" s="1" t="s">
+        <v>324</v>
+      </c>
       <c r="I392" s="23">
         <v>7106026</v>
       </c>
@@ -23428,7 +24013,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="393" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>1494</v>
+      </c>
       <c r="B393" t="s">
         <v>1279</v>
       </c>
@@ -23441,6 +24029,9 @@
       <c r="E393" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G393" s="1" t="s">
+        <v>324</v>
+      </c>
       <c r="I393" s="23">
         <v>7106027</v>
       </c>
@@ -23448,7 +24039,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="394" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
+        <v>1495</v>
+      </c>
       <c r="B394" t="s">
         <v>1279</v>
       </c>
@@ -23461,6 +24055,9 @@
       <c r="E394" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G394" s="1" t="s">
+        <v>327</v>
+      </c>
       <c r="I394" s="23">
         <v>7106028</v>
       </c>
@@ -23468,7 +24065,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="395" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A395" t="s">
+        <v>1496</v>
+      </c>
       <c r="B395" t="s">
         <v>1279</v>
       </c>
@@ -23481,6 +24081,9 @@
       <c r="E395" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G395" s="1" t="s">
+        <v>327</v>
+      </c>
       <c r="I395" s="23">
         <v>7106029</v>
       </c>
@@ -23488,7 +24091,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="396" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>1497</v>
+      </c>
       <c r="B396" t="s">
         <v>1279</v>
       </c>
@@ -23501,6 +24107,9 @@
       <c r="E396" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G396" s="1" t="s">
+        <v>331</v>
+      </c>
       <c r="I396" s="23">
         <v>7106030</v>
       </c>
@@ -23508,7 +24117,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="397" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>1498</v>
+      </c>
       <c r="B397" t="s">
         <v>1279</v>
       </c>
@@ -23521,6 +24133,9 @@
       <c r="E397" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G397" s="1" t="s">
+        <v>331</v>
+      </c>
       <c r="I397" s="23">
         <v>7106031</v>
       </c>
@@ -23528,7 +24143,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="398" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A398" t="s">
+        <v>1499</v>
+      </c>
       <c r="B398" t="s">
         <v>1279</v>
       </c>
@@ -23541,6 +24159,9 @@
       <c r="E398" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G398" s="1" t="s">
+        <v>334</v>
+      </c>
       <c r="I398" s="23">
         <v>7106032</v>
       </c>
@@ -23548,7 +24169,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="399" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A399" t="s">
+        <v>1500</v>
+      </c>
       <c r="B399" t="s">
         <v>1279</v>
       </c>
@@ -23561,6 +24185,9 @@
       <c r="E399" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G399" s="1" t="s">
+        <v>334</v>
+      </c>
       <c r="I399" s="23">
         <v>7106033</v>
       </c>
@@ -23568,7 +24195,10 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="400" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A400" t="s">
+        <v>1501</v>
+      </c>
       <c r="B400" t="s">
         <v>1279</v>
       </c>
@@ -23581,6 +24211,9 @@
       <c r="E400" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G400" s="1" t="s">
+        <v>334</v>
+      </c>
       <c r="I400" s="23">
         <v>7106034</v>
       </c>
@@ -23589,6 +24222,9 @@
       </c>
     </row>
     <row r="401" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A401" t="s">
+        <v>1502</v>
+      </c>
       <c r="B401" t="s">
         <v>1279</v>
       </c>
@@ -23601,6 +24237,9 @@
       <c r="E401" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G401" s="1" t="s">
+        <v>338</v>
+      </c>
       <c r="I401" s="23">
         <v>7106035</v>
       </c>
@@ -23609,6 +24248,9 @@
       </c>
     </row>
     <row r="402" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>1503</v>
+      </c>
       <c r="B402" t="s">
         <v>1279</v>
       </c>
@@ -23621,6 +24263,9 @@
       <c r="E402" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G402" s="1" t="s">
+        <v>338</v>
+      </c>
       <c r="I402" s="23">
         <v>7106036</v>
       </c>
@@ -23629,6 +24274,9 @@
       </c>
     </row>
     <row r="403" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>1504</v>
+      </c>
       <c r="B403" t="s">
         <v>1279</v>
       </c>
@@ -23641,6 +24289,9 @@
       <c r="E403" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G403" s="1" t="s">
+        <v>338</v>
+      </c>
       <c r="I403" s="23">
         <v>7106037</v>
       </c>
@@ -23649,6 +24300,9 @@
       </c>
     </row>
     <row r="404" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>1505</v>
+      </c>
       <c r="B404" t="s">
         <v>1279</v>
       </c>
@@ -23661,6 +24315,9 @@
       <c r="E404" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G404" s="1" t="s">
+        <v>1516</v>
+      </c>
       <c r="I404" s="23">
         <v>7106038</v>
       </c>
@@ -23669,6 +24326,9 @@
       </c>
     </row>
     <row r="405" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>1506</v>
+      </c>
       <c r="B405" t="s">
         <v>1279</v>
       </c>
@@ -23681,6 +24341,9 @@
       <c r="E405" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G405" s="1" t="s">
+        <v>1516</v>
+      </c>
       <c r="I405" s="23">
         <v>7106039</v>
       </c>
@@ -23689,6 +24352,9 @@
       </c>
     </row>
     <row r="406" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>1507</v>
+      </c>
       <c r="B406" t="s">
         <v>1279</v>
       </c>
@@ -23701,6 +24367,9 @@
       <c r="E406" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G406" s="1" t="s">
+        <v>1516</v>
+      </c>
       <c r="I406" s="23">
         <v>7106040</v>
       </c>
@@ -23709,6 +24378,9 @@
       </c>
     </row>
     <row r="407" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>1508</v>
+      </c>
       <c r="B407" t="s">
         <v>1279</v>
       </c>
@@ -23721,6 +24393,9 @@
       <c r="E407" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G407" s="1" t="s">
+        <v>345</v>
+      </c>
       <c r="I407" s="23">
         <v>7106041</v>
       </c>
@@ -23729,6 +24404,9 @@
       </c>
     </row>
     <row r="408" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>1509</v>
+      </c>
       <c r="B408" t="s">
         <v>1279</v>
       </c>
@@ -23741,6 +24419,9 @@
       <c r="E408" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G408" s="1" t="s">
+        <v>345</v>
+      </c>
       <c r="I408" s="23">
         <v>7106042</v>
       </c>
@@ -23749,6 +24430,9 @@
       </c>
     </row>
     <row r="409" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>1510</v>
+      </c>
       <c r="B409" t="s">
         <v>1279</v>
       </c>
@@ -23761,6 +24445,9 @@
       <c r="E409" s="1" t="s">
         <v>62</v>
       </c>
+      <c r="G409" s="1" t="s">
+        <v>345</v>
+      </c>
       <c r="I409" s="23">
         <v>7106043</v>
       </c>
@@ -23769,34 +24456,43 @@
       </c>
     </row>
     <row r="410" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>144</v>
+      </c>
       <c r="B410" t="s">
-        <v>1279</v>
+        <v>602</v>
       </c>
       <c r="C410" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D410" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E410" s="1" t="s">
-        <v>62</v>
+        <v>506</v>
+      </c>
+      <c r="E410" t="s">
+        <v>1281</v>
+      </c>
+      <c r="F410" t="s">
+        <v>143</v>
+      </c>
+      <c r="H410" t="s">
+        <v>1282</v>
       </c>
       <c r="I410" s="23">
-        <v>7106044</v>
+        <v>7101042</v>
       </c>
       <c r="L410" s="1" t="s">
-        <v>1280</v>
+        <v>658</v>
       </c>
     </row>
     <row r="411" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="B411" t="s">
         <v>602</v>
       </c>
       <c r="C411" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D411" s="1" t="s">
         <v>506</v>
@@ -23805,27 +24501,27 @@
         <v>1281</v>
       </c>
       <c r="F411" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="H411" t="s">
         <v>1282</v>
       </c>
-      <c r="I411" s="23">
-        <v>7101042</v>
+      <c r="I411" s="22">
+        <v>7102005</v>
       </c>
       <c r="L411" s="1" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="412" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>158</v>
+        <v>213</v>
       </c>
       <c r="B412" t="s">
         <v>602</v>
       </c>
       <c r="C412" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D412" s="1" t="s">
         <v>506</v>
@@ -23834,27 +24530,30 @@
         <v>1281</v>
       </c>
       <c r="F412" t="s">
-        <v>156</v>
+        <v>211</v>
       </c>
       <c r="H412" t="s">
         <v>1282</v>
       </c>
-      <c r="I412" s="22">
-        <v>7102005</v>
+      <c r="I412" s="23">
+        <v>7103001</v>
+      </c>
+      <c r="K412" s="1" t="s">
+        <v>1283</v>
       </c>
       <c r="L412" s="1" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="413" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>213</v>
+        <v>294</v>
       </c>
       <c r="B413" t="s">
         <v>602</v>
       </c>
       <c r="C413" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D413" s="1" t="s">
         <v>506</v>
@@ -23863,62 +24562,31 @@
         <v>1281</v>
       </c>
       <c r="F413" t="s">
-        <v>211</v>
+        <v>293</v>
       </c>
       <c r="H413" t="s">
         <v>1282</v>
       </c>
       <c r="I413" s="23">
-        <v>7103001</v>
-      </c>
-      <c r="K413" s="1" t="s">
-        <v>1283</v>
+        <v>7104001</v>
       </c>
       <c r="L413" s="1" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="414" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A414" t="s">
-        <v>294</v>
-      </c>
-      <c r="B414" t="s">
-        <v>602</v>
-      </c>
-      <c r="C414" t="s">
-        <v>41</v>
-      </c>
-      <c r="D414" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="E414" t="s">
-        <v>1281</v>
-      </c>
-      <c r="F414" t="s">
-        <v>293</v>
-      </c>
-      <c r="H414" t="s">
-        <v>1282</v>
-      </c>
-      <c r="I414" s="23">
-        <v>7104001</v>
-      </c>
-      <c r="L414" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:K493" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A2:K492" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="C3:C500" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C3:C499" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Relic,Weapon,Clue,Tarot Cards,Augmentation,Work of Mercy upgrade,Key Item / Skill,EXP Statue,Trap"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H3:H500" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H3:H499" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B3:B500" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B3:B499" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Silver Chest,Gold Chest,Unique Reward,Ghost,Statue,Note / Stele,Absorption (Boss/NPC),Augmentation (walk over),Augmentation (interact),Work of Mercy,Scripted Event,Interaction (Weapon),Destruction (Statue),Other"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -25272,24 +25940,22 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="36" customWidth="1"/>
-    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="2" max="2" width="40" style="1" customWidth="1"/>
+    <col min="3" max="5" width="30.7109375" customWidth="1"/>
+    <col min="6" max="6" width="36" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>1424</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>1425</v>
       </c>
@@ -25309,18 +25975,902 @@
         <v>1430</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>1431</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>1432</v>
-      </c>
-      <c r="I2" s="8" t="s">
         <v>58</v>
       </c>
     </row>
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>1517</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>1560</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>1561</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>1562</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>1563</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1470</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>1520</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>1521</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>1564</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>1565</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>1566</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1472</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>1523</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1474</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>1524</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>1567</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>1568</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>1569</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>1525</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1476</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>1526</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F12" t="s">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>1570</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>1571</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>1529</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>1572</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>1573</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>1574</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F16" t="s">
+        <v>1481</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>1531</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>1532</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>1575</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>1576</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>1577</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1483</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>1533</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1485</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>1535</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>1578</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>1579</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>1580</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>1536</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1487</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>1537</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>1538</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>1581</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>1582</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>1583</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1489</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>1540</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>1541</v>
+      </c>
+      <c r="C27" s="24" t="s">
+        <v>1584</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>1585</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>1586</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>1542</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>1543</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F29" t="s">
+        <v>1494</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>1544</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>1587</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>1588</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F30" t="s">
+        <v>1495</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>1545</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>1546</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>1589</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>1590</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1498</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>1548</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>1591</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>1592</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>1593</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1500</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>1550</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B37" s="19" t="s">
+        <v>1551</v>
+      </c>
+      <c r="C37" s="24" t="s">
+        <v>1594</v>
+      </c>
+      <c r="D37" s="24" t="s">
+        <v>1595</v>
+      </c>
+      <c r="E37" s="24" t="s">
+        <v>1596</v>
+      </c>
+      <c r="F37" t="s">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>1552</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F38" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>1553</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E39" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F39" t="s">
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>1554</v>
+      </c>
+      <c r="C40" s="24" t="s">
+        <v>1597</v>
+      </c>
+      <c r="D40" s="24" t="s">
+        <v>1598</v>
+      </c>
+      <c r="E40" s="24" t="s">
+        <v>1599</v>
+      </c>
+      <c r="F40" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>1555</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>1556</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E42" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F42" t="s">
+        <v>1507</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>1557</v>
+      </c>
+      <c r="C43" s="24" t="s">
+        <v>1600</v>
+      </c>
+      <c r="D43" s="24" t="s">
+        <v>1601</v>
+      </c>
+      <c r="E43" s="24" t="s">
+        <v>1602</v>
+      </c>
+      <c r="F43" t="s">
+        <v>1508</v>
+      </c>
+      <c r="G43" s="18" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>1558</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F44" t="s">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>1559</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F45" t="s">
+        <v>1510</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:I499" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="A2:G499" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>